<commit_message>
Set load times to 05:00 morning, 14:00 day, 01:00 night across all Excel sheets
Co-authored-by: gltdelete-prog <gltdelete-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SERDECHNOV-TEAM-grafik-avgust-2026.xlsx
+++ b/SERDECHNOV-TEAM-grafik-avgust-2026.xlsx
@@ -571,20 +571,20 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>02:00
-(Маш.2)</t>
+          <t>01:00
+(Машина 2)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>06:00
-(Маш.1)</t>
+          <t>05:00
+(Машина 1)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>18:00
-(Маш.1)</t>
+          <t>14:00
+(Машина 1)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -2007,7 +2007,7 @@
       <c r="A39" s="13" t="n"/>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>02:00 — ночной рейс (Машина 2)</t>
+          <t>01:00 — ночной рейс (Машина 2)</t>
         </is>
       </c>
     </row>
@@ -2015,7 +2015,7 @@
       <c r="A40" s="15" t="n"/>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>06:00 / 18:00 — дневные рейсы (Машина 1, один водитель)</t>
+          <t>05:00 / 14:00 — дневные рейсы (Машина 1, один водитель)</t>
         </is>
       </c>
     </row>
@@ -2297,12 +2297,12 @@
       </c>
       <c r="B9" s="22" t="inlineStr">
         <is>
-          <t>02:00 (ночь)</t>
+          <t>01:00 (ночь)</t>
         </is>
       </c>
       <c r="C9" s="22" t="inlineStr">
         <is>
-          <t>06:00 + 18:00 (день)</t>
+          <t>05:00 + 14:00 (день)</t>
         </is>
       </c>
     </row>
@@ -2389,7 +2389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2436,7 +2436,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -2463,17 +2463,17 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>01:30</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Выезд на ночную загрузку</t>
+          <t>Загрузка маршрут 7 (ночь)</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>≥ 1300</t>
+          <t>1341</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -2490,66 +2490,66 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Загрузка маршрут 7</t>
+          <t>Проверить ШК перед утренней загрузкой</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>1341</t>
+          <t>≥ 1300</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Машина 2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Ночной водитель</t>
+          <t>Дежурный ПВЗ</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>05:00</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Проверить ШК перед утренней загрузкой</t>
+          <t>Загрузка маршрут 7 (утро)</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>≥ 1300</t>
+          <t>1341</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Машина 1</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Дежурный ПВЗ</t>
+          <t>Дневной водитель</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Выезд на утреннюю загрузку</t>
+          <t>Проверить ШК перед дневной загрузкой</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -2559,24 +2559,24 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Машина 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>Дневной водитель</t>
+          <t>Дежурный ПВЗ</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Загрузка маршрут 7</t>
+          <t>Загрузка маршрут 7 (день)</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -2590,87 +2590,6 @@
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Дневной водитель</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Проверить ШК перед вечерней загрузкой</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>≥ 1300</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Дежурный ПВЗ</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Выезд на вечернюю загрузку</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>≥ 1300</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Машина 1</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>Дневной водитель</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Загрузка маршрут 7</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>1341</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Машина 1</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>Дневной водитель</t>
         </is>

</xml_diff>